<commit_message>
synthesis: close non-function conformance lanes and stage function-definition handoff
</commit_message>
<xml_diff>
--- a/research/runs/20260228-180047-excel-compat-empirical-pass-01/fixtures/table_wave1/SCN-EB034-STRUCTREF-SPILL.xlsx
+++ b/research/runs/20260228-180047-excel-compat-empirical-pass-01/fixtures/table_wave1/SCN-EB034-STRUCTREF-SPILL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Work\DnaCalc\Foundation\research\runs\20260228-180047-excel-compat-empirical-pass-01\fixtures\table_wave1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C33FB282-8237-46FC-9AD6-66F3B6AFDD1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11030B78-73B8-43AC-873D-8B11EA9F431A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3135" yWindow="3885" windowWidth="11955" windowHeight="11595" xr2:uid="{2E202768-54D3-4716-97D5-C413C3875489}"/>
   </bookViews>
@@ -101,9 +101,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -535,15 +534,15 @@
       <c r="B4">
         <v>3</v>
       </c>
-      <c r="C4" s="1">
+      <c r="C4">
         <f>TblMain[[#This Row],[Val]]*2</f>
         <v>6</v>
       </c>
-      <c r="D4" s="1">
+      <c r="D4">
         <f>SUM(TblMain[Val])</f>
         <v>6</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4">
         <f>_xlfn.SEQUENCE(ROWS(TblMain[Val]),1,1,1)</f>
         <v>1</v>
       </c>

</xml_diff>